<commit_message>
Soupisy: výkon těles potvrzen na kus, doplněn celkový výkon (počet × výkon)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9BziDSBzJTVtPM6bhxvYE
</commit_message>
<xml_diff>
--- a/vystupy/1OG_soupis_z_PDF.xlsx
+++ b/vystupy/1OG_soupis_z_PDF.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Párováno k nejbližšímu popisku 'P ≈ … W' (typicky 750 mm pod názvem; vzdálenost uvedena pro kontrolu). U '3x …' NENÍ ověřeno, zda výkon platí na kus, nebo celkem.</t>
+          <t>Párováno k nejbližšímu popisku 'P ≈ … W'. POTVRZENO (uživatel, 2026-10-06): výkon v popisku platí na 1 kus; u '3x …' je celkový výkon = počet × výkon. Viz sloupec 'Výkon celkem W'.</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Výkon W (nejbližší popisek P≈)</t>
+          <t>Výkon W na 1 kus (potvrzeno uživatelem)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -652,6 +652,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Jistota párování výkonu</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Výkon celkem W (počet × výkon/ks)</t>
         </is>
       </c>
     </row>
@@ -686,6 +691,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I2" t="n">
+        <v>3200</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -718,6 +726,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I3" t="n">
+        <v>2300</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -750,6 +761,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I4" t="n">
+        <v>1500</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -782,6 +796,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I5" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -814,6 +831,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I6" t="n">
+        <v>1600</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -846,6 +866,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I7" t="n">
+        <v>1100</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -878,6 +901,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I8" t="n">
+        <v>2400</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -910,6 +936,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I9" t="n">
+        <v>5100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -942,6 +971,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I10" t="n">
+        <v>16500</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -974,6 +1006,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I11" t="n">
+        <v>23100</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1006,6 +1041,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I12" t="n">
+        <v>3600</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1038,6 +1076,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I13" t="n">
+        <v>1600</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1070,6 +1111,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I14" t="n">
+        <v>1600</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1102,6 +1146,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I15" t="n">
+        <v>1200</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1134,6 +1181,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I16" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1166,6 +1216,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I17" t="n">
+        <v>11400</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1198,6 +1251,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I18" t="n">
+        <v>2800</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1230,6 +1286,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I19" t="n">
+        <v>350</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1262,6 +1321,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I20" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1294,6 +1356,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I21" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1326,6 +1391,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I22" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1357,6 +1425,9 @@
         <is>
           <t>OVĚŘIT ve výkresu</t>
         </is>
+      </c>
+      <c r="I23" t="n">
+        <v>7700</v>
       </c>
     </row>
     <row r="24">
@@ -1418,6 +1489,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I25" t="n">
+        <v>5775</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1450,6 +1524,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I26" t="n">
+        <v>18000</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1482,6 +1559,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I27" t="n">
+        <v>1200</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1514,6 +1594,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I28" t="n">
+        <v>3800</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1546,6 +1629,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I29" t="n">
+        <v>550</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1578,6 +1664,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I30" t="n">
+        <v>3500</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1610,6 +1699,9 @@
           <t>OVĚŘIT ve výkresu</t>
         </is>
       </c>
+      <c r="I31" t="n">
+        <v>1400</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1641,6 +1733,9 @@
         <is>
           <t>OVĚŘIT ve výkresu</t>
         </is>
+      </c>
+      <c r="I32" t="n">
+        <v>1900</v>
       </c>
     </row>
     <row r="33">
@@ -1702,6 +1797,9 @@
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
       </c>
+      <c r="I34" t="n">
+        <v>1200</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1733,6 +1831,9 @@
         <is>
           <t>OK (popisek 0,73 m pod názvem)</t>
         </is>
+      </c>
+      <c r="I35" t="n">
+        <v>1300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>